<commit_message>
allow empty phone number
</commit_message>
<xml_diff>
--- a/data/hotel_data.xlsx
+++ b/data/hotel_data.xlsx
@@ -1,26 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30015"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30023"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_03FADC941F5B28BEE64AD4174E5DCE3A074CA1E4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_03FADC941F5B28BEE64AD4174E5DCE3A074CA1E4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BDEA01EA-4B5C-4741-9424-5B3EDEBE01CB}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Contacten" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="271">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="269">
   <si>
     <t>Achternaam</t>
   </si>
@@ -824,12 +835,6 @@
   </si>
   <si>
     <t>0613278320</t>
-  </si>
-  <si>
-    <t>luuk.degroot@example.com</t>
-  </si>
-  <si>
-    <t>0619774839</t>
   </si>
   <si>
     <t>eva.beek@testmail.org</t>
@@ -2910,9 +2915,6 @@
       <c r="D100" t="s">
         <v>267</v>
       </c>
-      <c r="E100" t="s">
-        <v>268</v>
-      </c>
     </row>
     <row r="101" spans="1:5">
       <c r="A101" t="s">
@@ -2924,11 +2926,8 @@
       <c r="C101" s="2">
         <v>313</v>
       </c>
-      <c r="D101" t="s">
-        <v>269</v>
-      </c>
       <c r="E101" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
     </row>
   </sheetData>

</xml_diff>